<commit_message>
tests + new datasets
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_Bagging_kmeans_regression.xlsx
+++ b/output/reports/cv_experiment_Bagging_kmeans_regression.xlsx
@@ -491,23 +491,23 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>1.4497971534729</v>
+        <v>1.937947750091553</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9993661750125149</v>
+        <v>0.9916672509648135</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9997201460968009</v>
+        <v>0.9926310374474091</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3296664859921038</v>
+        <v>1.691656918987547</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2273045995670993</v>
+        <v>1.079954545454545</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'max_features': 0.8, 'max_samples': 1.0, 'n_estimators': 100}</t>
+          <t>{'max_features': 1.0, 'max_samples': 1.0, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -526,23 +526,23 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>2.304472208023071</v>
+        <v>2.616126298904419</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9994024065876171</v>
+        <v>0.991944820007945</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9997201460968009</v>
+        <v>0.9924359336701404</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3296664859921038</v>
+        <v>1.713905130730069</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2273045995670993</v>
+        <v>1.105564935064935</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'max_features': 0.8, 'max_samples': 1.0, 'n_estimators': 100}</t>
+          <t>{'max_features': 1.0, 'max_samples': 0.8, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -622,23 +622,23 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>1.4497971534729</v>
+        <v>1.937947750091553</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9993661750125149</v>
+        <v>0.9916672509648135</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9997201460968009</v>
+        <v>0.9926310374474091</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3296664859921038</v>
+        <v>1.691656918987547</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2273045995670993</v>
+        <v>1.079954545454545</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'max_features': 0.8, 'max_samples': 1.0, 'n_estimators': 100}</t>
+          <t>{'max_features': 1.0, 'max_samples': 1.0, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -657,23 +657,23 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>2.304472208023071</v>
+        <v>2.616126298904419</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9994024065876171</v>
+        <v>0.991944820007945</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9997201460968009</v>
+        <v>0.9924359336701404</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3296664859921038</v>
+        <v>1.713905130730069</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2273045995670993</v>
+        <v>1.105564935064935</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'max_features': 0.8, 'max_samples': 1.0, 'n_estimators': 100}</t>
+          <t>{'max_features': 1.0, 'max_samples': 0.8, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add visualizaion graphs for CV search
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_Bagging_kmeans_regression.xlsx
+++ b/output/reports/cv_experiment_Bagging_kmeans_regression.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,13 +488,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="D2" t="n">
-        <v>20.71422243118286</v>
+        <v>773.1986422538757</v>
       </c>
       <c r="E2" t="n">
-        <v>0.944157492185361</v>
+        <v>0.9503921749831643</v>
       </c>
       <c r="F2" t="n">
         <v>0.949013231773535</v>
@@ -523,13 +523,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="D3" t="n">
-        <v>39.83931756019592</v>
+        <v>115.5476741790771</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9469375966432583</v>
+        <v>0.9497617034790053</v>
       </c>
       <c r="F3" t="n">
         <v>0.949013231773535</v>
@@ -543,41 +543,6 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>{'max_features': 1.0, 'max_samples': 1.0, 'n_estimators': 100}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Bagging</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D4" t="n">
-        <v>86.38496446609497</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.9491455793684336</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.9499988975446574</v>
-      </c>
-      <c r="G4" t="n">
-        <v>39.7907712481769</v>
-      </c>
-      <c r="H4" t="n">
-        <v>23.77624280782508</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>{'max_features': 1.0, 'max_samples': 0.8, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -592,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -654,13 +619,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="D2" t="n">
-        <v>20.71422243118286</v>
+        <v>773.1986422538757</v>
       </c>
       <c r="E2" t="n">
-        <v>0.944157492185361</v>
+        <v>0.9503921749831643</v>
       </c>
       <c r="F2" t="n">
         <v>0.949013231773535</v>
@@ -689,13 +654,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="D3" t="n">
-        <v>39.83931756019592</v>
+        <v>115.5476741790771</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9469375966432583</v>
+        <v>0.9497617034790053</v>
       </c>
       <c r="F3" t="n">
         <v>0.949013231773535</v>
@@ -709,41 +674,6 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>{'max_features': 1.0, 'max_samples': 1.0, 'n_estimators': 100}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Bagging</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D4" t="n">
-        <v>86.38496446609497</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.9491455793684336</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.9499988975446574</v>
-      </c>
-      <c r="G4" t="n">
-        <v>39.7907712481769</v>
-      </c>
-      <c r="H4" t="n">
-        <v>23.77624280782508</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>{'max_features': 1.0, 'max_samples': 0.8, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>

</xml_diff>